<commit_message>
deposit and offline deposit bug fixed
</commit_message>
<xml_diff>
--- a/server/static/sample_file.xlsx
+++ b/server/static/sample_file.xlsx
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Atestertdhe</t>
+          <t>Atesterk4bj</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -489,7 +489,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Atestertdhe</t>
+          <t>Atesterk4bj</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -515,7 +515,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Atestertdhe</t>
+          <t>Atesterk4bj</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -541,7 +541,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Atestertdhe</t>
+          <t>Atesterk4bj</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -567,7 +567,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Atestertdhe</t>
+          <t>Atesterk4bj</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -593,7 +593,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Atestertdhe</t>
+          <t>Atesterk4bj</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>

</xml_diff>